<commit_message>
after edit image subcategories
</commit_message>
<xml_diff>
--- a/Back-End-Laravel/database/seeders/data/products.xlsx
+++ b/Back-End-Laravel/database/seeders/data/products.xlsx
@@ -1038,6 +1038,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:H111"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1077,7 +1078,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
@@ -1094,7 +1095,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>13</v>
       </c>
@@ -1111,7 +1112,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>15</v>
       </c>
@@ -1128,7 +1129,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>17</v>
       </c>
@@ -1145,7 +1146,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>19</v>
       </c>
@@ -1162,7 +1163,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>21</v>
       </c>
@@ -1179,7 +1180,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>23</v>
       </c>
@@ -1196,7 +1197,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>25</v>
       </c>
@@ -1213,7 +1214,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>27</v>
       </c>
@@ -1230,7 +1231,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>29</v>
       </c>
@@ -1247,7 +1248,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>31</v>
       </c>
@@ -1264,7 +1265,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>33</v>
       </c>
@@ -1281,7 +1282,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>35</v>
       </c>
@@ -1298,7 +1299,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>37</v>
       </c>
@@ -1315,7 +1316,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>39</v>
       </c>
@@ -1332,7 +1333,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>41</v>
       </c>
@@ -1349,7 +1350,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>43</v>
       </c>
@@ -1366,7 +1367,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>45</v>
       </c>
@@ -1383,7 +1384,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>47</v>
       </c>
@@ -1400,7 +1401,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>49</v>
       </c>
@@ -1417,7 +1418,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>51</v>
       </c>
@@ -1434,7 +1435,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>53</v>
       </c>
@@ -1451,7 +1452,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>55</v>
       </c>
@@ -1468,7 +1469,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>57</v>
       </c>
@@ -1485,7 +1486,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>59</v>
       </c>
@@ -1502,7 +1503,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>61</v>
       </c>
@@ -1519,7 +1520,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>63</v>
       </c>
@@ -1536,7 +1537,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>65</v>
       </c>
@@ -1553,7 +1554,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>67</v>
       </c>
@@ -1570,7 +1571,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>69</v>
       </c>
@@ -1587,7 +1588,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>71</v>
       </c>
@@ -1604,7 +1605,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>73</v>
       </c>
@@ -1621,7 +1622,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>75</v>
       </c>
@@ -1638,7 +1639,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>77</v>
       </c>
@@ -1655,7 +1656,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>79</v>
       </c>
@@ -1672,7 +1673,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>81</v>
       </c>
@@ -1689,7 +1690,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>83</v>
       </c>
@@ -1706,7 +1707,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>85</v>
       </c>
@@ -1723,7 +1724,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>87</v>
       </c>
@@ -1740,7 +1741,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>89</v>
       </c>
@@ -1757,7 +1758,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>91</v>
       </c>
@@ -1774,7 +1775,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>93</v>
       </c>
@@ -1791,7 +1792,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>95</v>
       </c>
@@ -1808,7 +1809,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>97</v>
       </c>
@@ -1825,7 +1826,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>99</v>
       </c>
@@ -1842,7 +1843,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>101</v>
       </c>
@@ -1859,7 +1860,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>103</v>
       </c>
@@ -1876,7 +1877,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>105</v>
       </c>
@@ -1893,7 +1894,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>107</v>
       </c>
@@ -1910,7 +1911,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>109</v>
       </c>
@@ -1927,7 +1928,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>111</v>
       </c>
@@ -1944,7 +1945,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>113</v>
       </c>
@@ -1961,7 +1962,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>115</v>
       </c>
@@ -1978,7 +1979,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
         <v>117</v>
       </c>
@@ -1995,7 +1996,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>119</v>
       </c>
@@ -2012,7 +2013,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>121</v>
       </c>
@@ -2029,7 +2030,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>123</v>
       </c>
@@ -2046,7 +2047,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>125</v>
       </c>
@@ -2063,7 +2064,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>127</v>
       </c>
@@ -2080,7 +2081,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
         <v>129</v>
       </c>
@@ -2097,7 +2098,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>131</v>
       </c>
@@ -2114,7 +2115,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
         <v>133</v>
       </c>
@@ -2131,7 +2132,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>135</v>
       </c>
@@ -2148,7 +2149,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>137</v>
       </c>
@@ -2165,7 +2166,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
         <v>139</v>
       </c>
@@ -2182,7 +2183,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
         <v>141</v>
       </c>
@@ -2199,7 +2200,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
         <v>143</v>
       </c>
@@ -2216,7 +2217,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
         <v>145</v>
       </c>
@@ -2233,7 +2234,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
         <v>147</v>
       </c>
@@ -2250,7 +2251,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
         <v>149</v>
       </c>
@@ -2267,7 +2268,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
         <v>151</v>
       </c>
@@ -2284,7 +2285,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
         <v>153</v>
       </c>
@@ -2301,7 +2302,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
         <v>155</v>
       </c>
@@ -2318,7 +2319,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
         <v>157</v>
       </c>
@@ -2335,7 +2336,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
         <v>159</v>
       </c>
@@ -2352,7 +2353,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
         <v>161</v>
       </c>
@@ -2529,7 +2530,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
         <v>179</v>
       </c>
@@ -2546,7 +2547,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87" s="1" t="s">
         <v>181</v>
       </c>
@@ -2563,7 +2564,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88" s="1" t="s">
         <v>183</v>
       </c>
@@ -2580,7 +2581,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89" s="1" t="s">
         <v>185</v>
       </c>
@@ -2597,7 +2598,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90" s="1" t="s">
         <v>187</v>
       </c>
@@ -2614,7 +2615,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
         <v>189</v>
       </c>
@@ -2631,7 +2632,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A92" s="1" t="s">
         <v>191</v>
       </c>
@@ -2648,7 +2649,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A93" s="1" t="s">
         <v>193</v>
       </c>
@@ -2665,7 +2666,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A94" s="1" t="s">
         <v>195</v>
       </c>
@@ -2682,7 +2683,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A95" s="1" t="s">
         <v>197</v>
       </c>
@@ -2699,7 +2700,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A96" s="1" t="s">
         <v>199</v>
       </c>
@@ -2716,7 +2717,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A97" s="1" t="s">
         <v>201</v>
       </c>
@@ -2733,7 +2734,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A98" s="1" t="s">
         <v>203</v>
       </c>
@@ -2750,7 +2751,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A99" s="1" t="s">
         <v>205</v>
       </c>
@@ -2767,7 +2768,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A100" s="1" t="s">
         <v>207</v>
       </c>
@@ -2784,7 +2785,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A101" s="1" t="s">
         <v>209</v>
       </c>
@@ -2801,7 +2802,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A102" s="1" t="s">
         <v>211</v>
       </c>
@@ -2818,7 +2819,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A103" s="1" t="s">
         <v>213</v>
       </c>
@@ -2835,7 +2836,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A104" s="1" t="s">
         <v>215</v>
       </c>
@@ -2852,7 +2853,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A105" s="1" t="s">
         <v>217</v>
       </c>
@@ -2869,7 +2870,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A106" s="1" t="s">
         <v>219</v>
       </c>
@@ -2886,7 +2887,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A107" s="1" t="s">
         <v>221</v>
       </c>
@@ -2903,7 +2904,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A108" s="1" t="s">
         <v>223</v>
       </c>
@@ -2920,7 +2921,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A109" s="1" t="s">
         <v>225</v>
       </c>
@@ -2937,7 +2938,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A110" s="1" t="s">
         <v>227</v>
       </c>
@@ -2954,7 +2955,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A111" s="1" t="s">
         <v>229</v>
       </c>
@@ -2972,7 +2973,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H111"/>
+  <autoFilter ref="A1:H111">
+    <filterColumn colId="7">
+      <customFilters>
+        <customFilter operator="notEqual" val=" "/>
+      </customFilters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
after edit pic in products
</commit_message>
<xml_diff>
--- a/Back-End-Laravel/database/seeders/data/products.xlsx
+++ b/Back-End-Laravel/database/seeders/data/products.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="566" uniqueCount="232">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="668" uniqueCount="235">
   <si>
     <t>code</t>
   </si>
@@ -718,6 +718,15 @@
   </si>
   <si>
     <t>products/tibial-base.png</t>
+  </si>
+  <si>
+    <t>products/tibial-liner.png</t>
+  </si>
+  <si>
+    <t>products/femoral-component.png</t>
+  </si>
+  <si>
+    <t>products/patella.png</t>
   </si>
 </sst>
 </file>
@@ -1038,7 +1047,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:H111"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1049,7 +1057,7 @@
     <col min="5" max="5" width="15.85546875" style="1" customWidth="1"/>
     <col min="6" max="6" width="18.85546875" style="1" customWidth="1"/>
     <col min="7" max="7" width="5.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="26.85546875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="32" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -1078,7 +1086,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
@@ -1094,8 +1102,11 @@
       <c r="F2" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H2" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>13</v>
       </c>
@@ -1111,8 +1122,11 @@
       <c r="F3" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H3" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>15</v>
       </c>
@@ -1128,8 +1142,11 @@
       <c r="F4" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H4" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>17</v>
       </c>
@@ -1145,8 +1162,11 @@
       <c r="F5" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H5" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>19</v>
       </c>
@@ -1162,8 +1182,11 @@
       <c r="F6" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H6" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>21</v>
       </c>
@@ -1179,8 +1202,11 @@
       <c r="F7" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H7" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>23</v>
       </c>
@@ -1196,8 +1222,11 @@
       <c r="F8" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H8" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>25</v>
       </c>
@@ -1213,8 +1242,11 @@
       <c r="F9" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H9" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>27</v>
       </c>
@@ -1230,8 +1262,11 @@
       <c r="F10" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H10" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>29</v>
       </c>
@@ -1247,8 +1282,11 @@
       <c r="F11" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H11" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>31</v>
       </c>
@@ -1264,8 +1302,11 @@
       <c r="F12" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H12" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>33</v>
       </c>
@@ -1281,8 +1322,11 @@
       <c r="F13" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H13" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>35</v>
       </c>
@@ -1298,8 +1342,11 @@
       <c r="F14" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H14" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>37</v>
       </c>
@@ -1315,8 +1362,11 @@
       <c r="F15" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H15" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>39</v>
       </c>
@@ -1332,8 +1382,11 @@
       <c r="F16" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H16" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>41</v>
       </c>
@@ -1349,8 +1402,11 @@
       <c r="F17" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H17" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>43</v>
       </c>
@@ -1366,8 +1422,11 @@
       <c r="F18" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H18" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>45</v>
       </c>
@@ -1383,8 +1442,11 @@
       <c r="F19" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H19" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>47</v>
       </c>
@@ -1400,8 +1462,11 @@
       <c r="F20" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H20" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>49</v>
       </c>
@@ -1417,8 +1482,11 @@
       <c r="F21" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H21" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>51</v>
       </c>
@@ -1434,8 +1502,11 @@
       <c r="F22" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="23" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H22" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>53</v>
       </c>
@@ -1451,8 +1522,11 @@
       <c r="F23" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H23" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>55</v>
       </c>
@@ -1468,8 +1542,11 @@
       <c r="F24" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="25" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H24" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>57</v>
       </c>
@@ -1485,8 +1562,11 @@
       <c r="F25" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="26" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H25" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>59</v>
       </c>
@@ -1502,8 +1582,11 @@
       <c r="F26" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="27" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H26" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>61</v>
       </c>
@@ -1519,8 +1602,11 @@
       <c r="F27" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="28" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H27" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>63</v>
       </c>
@@ -1536,8 +1622,11 @@
       <c r="F28" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="29" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H28" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>65</v>
       </c>
@@ -1553,8 +1642,11 @@
       <c r="F29" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="30" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H29" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>67</v>
       </c>
@@ -1570,8 +1662,11 @@
       <c r="F30" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="31" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H30" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>69</v>
       </c>
@@ -1587,8 +1682,11 @@
       <c r="F31" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="32" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H31" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>71</v>
       </c>
@@ -1604,8 +1702,11 @@
       <c r="F32" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="33" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H32" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>73</v>
       </c>
@@ -1621,8 +1722,11 @@
       <c r="F33" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="34" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H33" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>75</v>
       </c>
@@ -1638,8 +1742,11 @@
       <c r="F34" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="35" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H34" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>77</v>
       </c>
@@ -1655,8 +1762,11 @@
       <c r="F35" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="36" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H35" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>79</v>
       </c>
@@ -1672,8 +1782,11 @@
       <c r="F36" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="37" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H36" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>81</v>
       </c>
@@ -1689,8 +1802,11 @@
       <c r="F37" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="38" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H37" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>83</v>
       </c>
@@ -1706,8 +1822,11 @@
       <c r="F38" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="39" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H38" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>85</v>
       </c>
@@ -1723,8 +1842,11 @@
       <c r="F39" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="40" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H39" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>87</v>
       </c>
@@ -1740,8 +1862,11 @@
       <c r="F40" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="41" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H40" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>89</v>
       </c>
@@ -1757,8 +1882,11 @@
       <c r="F41" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="42" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H41" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>91</v>
       </c>
@@ -1774,8 +1902,11 @@
       <c r="F42" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="43" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H42" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>93</v>
       </c>
@@ -1791,8 +1922,11 @@
       <c r="F43" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="44" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H43" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>95</v>
       </c>
@@ -1808,8 +1942,11 @@
       <c r="F44" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="45" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H44" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>97</v>
       </c>
@@ -1825,8 +1962,11 @@
       <c r="F45" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="46" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H45" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>99</v>
       </c>
@@ -1842,8 +1982,11 @@
       <c r="F46" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="47" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H46" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>101</v>
       </c>
@@ -1859,8 +2002,11 @@
       <c r="F47" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="48" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H47" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>103</v>
       </c>
@@ -1876,8 +2022,11 @@
       <c r="F48" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="49" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H48" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>105</v>
       </c>
@@ -1893,8 +2042,11 @@
       <c r="F49" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="50" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H49" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>107</v>
       </c>
@@ -1910,8 +2062,11 @@
       <c r="F50" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="51" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H50" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>109</v>
       </c>
@@ -1927,8 +2082,11 @@
       <c r="F51" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="52" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H51" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>111</v>
       </c>
@@ -1944,8 +2102,11 @@
       <c r="F52" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="53" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H52" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>113</v>
       </c>
@@ -1961,8 +2122,11 @@
       <c r="F53" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="54" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H53" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>115</v>
       </c>
@@ -1978,8 +2142,11 @@
       <c r="F54" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="55" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H54" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
         <v>117</v>
       </c>
@@ -1995,8 +2162,11 @@
       <c r="F55" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="56" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H55" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>119</v>
       </c>
@@ -2012,8 +2182,11 @@
       <c r="F56" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="57" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H56" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>121</v>
       </c>
@@ -2029,8 +2202,11 @@
       <c r="F57" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="58" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H57" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>123</v>
       </c>
@@ -2046,8 +2222,11 @@
       <c r="F58" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="59" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H58" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>125</v>
       </c>
@@ -2063,8 +2242,11 @@
       <c r="F59" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="60" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H59" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>127</v>
       </c>
@@ -2080,8 +2262,11 @@
       <c r="F60" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="61" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H60" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
         <v>129</v>
       </c>
@@ -2097,8 +2282,11 @@
       <c r="F61" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="62" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H61" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>131</v>
       </c>
@@ -2114,8 +2302,11 @@
       <c r="F62" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="63" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H62" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
         <v>133</v>
       </c>
@@ -2131,8 +2322,11 @@
       <c r="F63" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="64" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H63" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>135</v>
       </c>
@@ -2148,8 +2342,11 @@
       <c r="F64" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="65" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H64" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>137</v>
       </c>
@@ -2165,8 +2362,11 @@
       <c r="F65" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="66" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H65" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
         <v>139</v>
       </c>
@@ -2182,8 +2382,11 @@
       <c r="F66" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="67" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H66" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
         <v>141</v>
       </c>
@@ -2199,8 +2402,11 @@
       <c r="F67" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="68" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H67" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
         <v>143</v>
       </c>
@@ -2216,8 +2422,11 @@
       <c r="F68" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="69" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H68" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
         <v>145</v>
       </c>
@@ -2233,8 +2442,11 @@
       <c r="F69" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="70" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H69" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
         <v>147</v>
       </c>
@@ -2250,8 +2462,11 @@
       <c r="F70" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="71" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H70" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
         <v>149</v>
       </c>
@@ -2267,8 +2482,11 @@
       <c r="F71" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="72" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H71" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
         <v>151</v>
       </c>
@@ -2284,8 +2502,11 @@
       <c r="F72" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="73" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H72" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
         <v>153</v>
       </c>
@@ -2301,8 +2522,11 @@
       <c r="F73" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="74" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H73" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
         <v>155</v>
       </c>
@@ -2318,8 +2542,11 @@
       <c r="F74" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="75" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H74" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
         <v>157</v>
       </c>
@@ -2335,8 +2562,11 @@
       <c r="F75" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="76" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H75" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
         <v>159</v>
       </c>
@@ -2352,8 +2582,11 @@
       <c r="F76" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="77" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H76" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
         <v>161</v>
       </c>
@@ -2368,6 +2601,9 @@
       </c>
       <c r="F77" s="1" t="s">
         <v>12</v>
+      </c>
+      <c r="H77" s="1" t="s">
+        <v>232</v>
       </c>
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.25">
@@ -2530,7 +2766,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="86" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
         <v>179</v>
       </c>
@@ -2546,8 +2782,11 @@
       <c r="F86" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="87" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H86" s="1" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A87" s="1" t="s">
         <v>181</v>
       </c>
@@ -2563,8 +2802,11 @@
       <c r="F87" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="88" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H87" s="1" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A88" s="1" t="s">
         <v>183</v>
       </c>
@@ -2580,8 +2822,11 @@
       <c r="F88" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="89" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H88" s="1" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A89" s="1" t="s">
         <v>185</v>
       </c>
@@ -2597,8 +2842,11 @@
       <c r="F89" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="90" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H89" s="1" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A90" s="1" t="s">
         <v>187</v>
       </c>
@@ -2614,8 +2862,11 @@
       <c r="F90" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="91" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H90" s="1" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
         <v>189</v>
       </c>
@@ -2631,8 +2882,11 @@
       <c r="F91" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="92" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H91" s="1" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A92" s="1" t="s">
         <v>191</v>
       </c>
@@ -2648,8 +2902,11 @@
       <c r="F92" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="93" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H92" s="1" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A93" s="1" t="s">
         <v>193</v>
       </c>
@@ -2665,8 +2922,11 @@
       <c r="F93" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="94" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H93" s="1" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A94" s="1" t="s">
         <v>195</v>
       </c>
@@ -2682,8 +2942,11 @@
       <c r="F94" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="95" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H94" s="1" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A95" s="1" t="s">
         <v>197</v>
       </c>
@@ -2699,8 +2962,11 @@
       <c r="F95" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="96" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H95" s="1" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A96" s="1" t="s">
         <v>199</v>
       </c>
@@ -2716,8 +2982,11 @@
       <c r="F96" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="97" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H96" s="1" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="97" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A97" s="1" t="s">
         <v>201</v>
       </c>
@@ -2733,8 +3002,11 @@
       <c r="F97" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="98" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H97" s="1" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="98" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A98" s="1" t="s">
         <v>203</v>
       </c>
@@ -2750,8 +3022,11 @@
       <c r="F98" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="99" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H98" s="1" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="99" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A99" s="1" t="s">
         <v>205</v>
       </c>
@@ -2767,8 +3042,11 @@
       <c r="F99" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="100" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H99" s="1" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="100" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A100" s="1" t="s">
         <v>207</v>
       </c>
@@ -2784,8 +3062,11 @@
       <c r="F100" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="101" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H100" s="1" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="101" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A101" s="1" t="s">
         <v>209</v>
       </c>
@@ -2801,8 +3082,11 @@
       <c r="F101" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="102" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H101" s="1" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="102" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A102" s="1" t="s">
         <v>211</v>
       </c>
@@ -2818,8 +3102,11 @@
       <c r="F102" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="103" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H102" s="1" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="103" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A103" s="1" t="s">
         <v>213</v>
       </c>
@@ -2835,8 +3122,11 @@
       <c r="F103" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="104" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H103" s="1" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="104" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A104" s="1" t="s">
         <v>215</v>
       </c>
@@ -2852,8 +3142,11 @@
       <c r="F104" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="105" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H104" s="1" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="105" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A105" s="1" t="s">
         <v>217</v>
       </c>
@@ -2869,8 +3162,11 @@
       <c r="F105" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="106" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H105" s="1" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="106" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A106" s="1" t="s">
         <v>219</v>
       </c>
@@ -2886,8 +3182,11 @@
       <c r="F106" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="107" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H106" s="1" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="107" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A107" s="1" t="s">
         <v>221</v>
       </c>
@@ -2903,8 +3202,11 @@
       <c r="F107" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="108" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H107" s="1" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="108" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A108" s="1" t="s">
         <v>223</v>
       </c>
@@ -2920,8 +3222,11 @@
       <c r="F108" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="109" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H108" s="1" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="109" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A109" s="1" t="s">
         <v>225</v>
       </c>
@@ -2937,8 +3242,11 @@
       <c r="F109" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="110" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H109" s="1" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="110" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A110" s="1" t="s">
         <v>227</v>
       </c>
@@ -2954,8 +3262,11 @@
       <c r="F110" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="111" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H110" s="1" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="111" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A111" s="1" t="s">
         <v>229</v>
       </c>
@@ -2971,15 +3282,12 @@
       <c r="F111" s="1" t="s">
         <v>12</v>
       </c>
+      <c r="H111" s="1" t="s">
+        <v>234</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H111">
-    <filterColumn colId="7">
-      <customFilters>
-        <customFilter operator="notEqual" val=" "/>
-      </customFilters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:H111"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
after add excel to operations
</commit_message>
<xml_diff>
--- a/Back-End-Laravel/database/seeders/data/products.xlsx
+++ b/Back-End-Laravel/database/seeders/data/products.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="668" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1406" uniqueCount="493">
   <si>
     <t>code</t>
   </si>
@@ -727,6 +727,780 @@
   </si>
   <si>
     <t>products/patella.png</t>
+  </si>
+  <si>
+    <t>MO-AOAC-10/35</t>
+  </si>
+  <si>
+    <t>Threading 3.5 mm hex drive Apical Hole Occluder M10</t>
+  </si>
+  <si>
+    <t>subcat-002</t>
+  </si>
+  <si>
+    <t>products/threading-3-5-mm-hex-drive-apical-hole-occluder-m10.png</t>
+  </si>
+  <si>
+    <t>MO-HDAA-22/00 12/14</t>
+  </si>
+  <si>
+    <t>CoCr Modular Femoral Head 22/0 Taper</t>
+  </si>
+  <si>
+    <t>products/cocr-modular-femoral-head-taper.png</t>
+  </si>
+  <si>
+    <t>MO-HDAA-22/35+12/14</t>
+  </si>
+  <si>
+    <t>CoCr Modular Femoral Head 22/+3.5 Taper</t>
+  </si>
+  <si>
+    <t>MO-HDAA-28/00 12/14</t>
+  </si>
+  <si>
+    <t>CoCr Modular Femoral Head 28/0 Taper</t>
+  </si>
+  <si>
+    <t>MO-HDAA-28/35+12/14</t>
+  </si>
+  <si>
+    <t>CoCr Modular Femoral Head 28/+3.5 Taper</t>
+  </si>
+  <si>
+    <t>MO-HDAA-28/35- 12/14</t>
+  </si>
+  <si>
+    <t>CoCr Modular Femoral Head 28/-3.5 Taper</t>
+  </si>
+  <si>
+    <t>MO-HDAA-28/70+ 12/14</t>
+  </si>
+  <si>
+    <t>CoCr Modular Femoral Head 28/+7 Taper</t>
+  </si>
+  <si>
+    <t>MO-HDAA-32/00 12/14</t>
+  </si>
+  <si>
+    <t>CoCr Modular Femoral Head 32/0 Taper</t>
+  </si>
+  <si>
+    <t>MO-HDAA-32/40+12/14</t>
+  </si>
+  <si>
+    <t>CoCr Modular Femoral Head 32/+4 Taper</t>
+  </si>
+  <si>
+    <t>MO-HDAA-32/40- 12/14</t>
+  </si>
+  <si>
+    <t>CoCr Modular Femoral Head 32/-4 Taper</t>
+  </si>
+  <si>
+    <t>MO-HDAA-32/70+ 12/14</t>
+  </si>
+  <si>
+    <t>CoCr Modular Femoral Head 32/+7 Taper</t>
+  </si>
+  <si>
+    <t>MO-HDAA-36/00 12/14</t>
+  </si>
+  <si>
+    <t>CoCr Modular Femoral Head 36/0 Taper</t>
+  </si>
+  <si>
+    <t>MO-HDAA-36/40+ 12/14</t>
+  </si>
+  <si>
+    <t>CoCr Modular Femoral Head 36/+4 Taper</t>
+  </si>
+  <si>
+    <t>MO-HDAA-36/40- 12/14</t>
+  </si>
+  <si>
+    <t>CoCr Modular Femoral Head 36/-4 Taper</t>
+  </si>
+  <si>
+    <t>MO-HDAA-36/70+ 12/14</t>
+  </si>
+  <si>
+    <t>CoCr Modular Femoral Head 36/+7 Taper</t>
+  </si>
+  <si>
+    <t>MO-HDAA-40/00 12/14</t>
+  </si>
+  <si>
+    <t>CoCr Modular Femoral Head 40/0 Taper</t>
+  </si>
+  <si>
+    <t>MO-HDAA-40/40+ 12/14</t>
+  </si>
+  <si>
+    <t>CoCr Modular Femoral Head 40/+4 Taper</t>
+  </si>
+  <si>
+    <t>MO-HDAA-40/40- 12/14</t>
+  </si>
+  <si>
+    <t>CoCr Modular Femoral Head 40/-4 Taper</t>
+  </si>
+  <si>
+    <t>MO-HDAA-40/70+ 12/14</t>
+  </si>
+  <si>
+    <t>CoCr Modular Femoral Head 40/+7 Taper</t>
+  </si>
+  <si>
+    <t>MO-HDAI-28/00 12/14</t>
+  </si>
+  <si>
+    <t>Modular Femoral Head  Biolox® Delta Ceramic 28/0 Taper</t>
+  </si>
+  <si>
+    <t>products/modular-femoral-head-biolox-delta-ceramic-taper.png</t>
+  </si>
+  <si>
+    <t>MO-HDAI-28/35+12/14</t>
+  </si>
+  <si>
+    <t>Modular Femoral Head  Biolox® Delta Ceramic 28/+3.5 Taper</t>
+  </si>
+  <si>
+    <t>MO-HDAI-28/35-12/14</t>
+  </si>
+  <si>
+    <t>Modular Femoral Head  Biolox® Delta Ceramic 28/-3.5 Taper</t>
+  </si>
+  <si>
+    <t>MO-HDAI-32/00 12/14</t>
+  </si>
+  <si>
+    <t>Modular Femoral Head  Biolox® Delta Ceramic 32/0 Taper</t>
+  </si>
+  <si>
+    <t>MO-HDAI-32/40+12/14</t>
+  </si>
+  <si>
+    <t>Modular Femoral Head  Biolox® Delta Ceramic 32/+4 Taper</t>
+  </si>
+  <si>
+    <t>MO-HDAI-32/40-12/14</t>
+  </si>
+  <si>
+    <t>Modular Femoral Head  Biolox® Delta Ceramic 32/-4 Taper</t>
+  </si>
+  <si>
+    <t>MO-HDAI-32/70+12/14</t>
+  </si>
+  <si>
+    <t>Modular Femoral Head  Biolox® Delta Ceramic 32/+7 Taper</t>
+  </si>
+  <si>
+    <t>MO-HDAI-36/00 12/14</t>
+  </si>
+  <si>
+    <t>Modular Femoral Head  Biolox® Delta Ceramic 36/0 Taper</t>
+  </si>
+  <si>
+    <t>MO-HDAI-36/40+12/14</t>
+  </si>
+  <si>
+    <t>Modular Femoral Head  Biolox® Delta Ceramic 36/+4 Taper</t>
+  </si>
+  <si>
+    <t>MO-HDAI-36/40-12/14</t>
+  </si>
+  <si>
+    <t>Modular Femoral Head  Biolox® Delta Ceramic 36/-4 Taper</t>
+  </si>
+  <si>
+    <t>MO-HDAI-36/80+12/14</t>
+  </si>
+  <si>
+    <t>Modular Femoral Head  Biolox® Delta Ceramic 36/+8 Taper</t>
+  </si>
+  <si>
+    <t>MO-HDAI-40/00 12/14</t>
+  </si>
+  <si>
+    <t>Modular Femoral Head  Biolox® Delta Ceramic 40/0 Taper</t>
+  </si>
+  <si>
+    <t>MO-HDAI-40/40+12/14</t>
+  </si>
+  <si>
+    <t>Modular Femoral Head  Biolox® Delta Ceramic 40/+4 Taper</t>
+  </si>
+  <si>
+    <t>MO-HDAI-40/40-12/14</t>
+  </si>
+  <si>
+    <t>Modular Femoral Head  Biolox® Delta Ceramic 40/-4 Taper</t>
+  </si>
+  <si>
+    <t>MO-HDAI-40/80+12/14</t>
+  </si>
+  <si>
+    <t>Modular Femoral Head  Biolox® Delta Ceramic 40/+8 Taper</t>
+  </si>
+  <si>
+    <t>MO-MLJE-MA/22</t>
+  </si>
+  <si>
+    <t>Modular Liner Size MA/22 10° Oblique</t>
+  </si>
+  <si>
+    <t>products/modular-liner-10-degree-oblique.png</t>
+  </si>
+  <si>
+    <t>MO-MLJE-MB/22</t>
+  </si>
+  <si>
+    <t>Modular Liner Size MB/22 10° Oblique</t>
+  </si>
+  <si>
+    <t>MO-MLJE-MB/28</t>
+  </si>
+  <si>
+    <t>Modular Liner Size MB/28 10° Oblique</t>
+  </si>
+  <si>
+    <t>MO-MLJE-MD/28</t>
+  </si>
+  <si>
+    <t>Modular Liner Size MD/28 10° Oblique</t>
+  </si>
+  <si>
+    <t>MO-MLJE-MD/32</t>
+  </si>
+  <si>
+    <t>Modular Liner Size MD/32 10° Oblique</t>
+  </si>
+  <si>
+    <t>MO-MLJE-MF/28</t>
+  </si>
+  <si>
+    <t>Modular Liner Size MF/28 10° Oblique</t>
+  </si>
+  <si>
+    <t>MO-MLJE-MF/32</t>
+  </si>
+  <si>
+    <t>Modular Liner Size MF/32 10° Oblique</t>
+  </si>
+  <si>
+    <t>MO-MLJE-MF/36</t>
+  </si>
+  <si>
+    <t>Modular Liner Size MF/36 10° Oblique</t>
+  </si>
+  <si>
+    <t>MO-MLJE-MH/28</t>
+  </si>
+  <si>
+    <t>Modular Liner Size MH/28 10° Oblique</t>
+  </si>
+  <si>
+    <t>MO-MLJE-MH/32</t>
+  </si>
+  <si>
+    <t>Modular Liner Size MH/32 10° Oblique</t>
+  </si>
+  <si>
+    <t>MO-MLJE-MH/36</t>
+  </si>
+  <si>
+    <t>Modular Liner Size MH/36 10° Oblique</t>
+  </si>
+  <si>
+    <t>MO-MLJE-MJ/32</t>
+  </si>
+  <si>
+    <t>Modular Liner Size MJ/32 10° Oblique</t>
+  </si>
+  <si>
+    <t>MO-MLJE-MJ/36</t>
+  </si>
+  <si>
+    <t>Modular Liner Size MJ/36 10° Oblique</t>
+  </si>
+  <si>
+    <t>MO-MLJE-MJ/40</t>
+  </si>
+  <si>
+    <t>Modular Liner Size MJ/40 10° Oblique</t>
+  </si>
+  <si>
+    <t>MO-MLJE-MK/32</t>
+  </si>
+  <si>
+    <t>Modular Liner Size MK/32 10° Oblique</t>
+  </si>
+  <si>
+    <t>MO-MLJE-MK/36</t>
+  </si>
+  <si>
+    <t>Modular Liner Size MK/36 10° Oblique</t>
+  </si>
+  <si>
+    <t>MO-MLJE-MK/40</t>
+  </si>
+  <si>
+    <t>Modular Liner Size MK/40 10° Oblique</t>
+  </si>
+  <si>
+    <t>MO-MLLE-MA/22 </t>
+  </si>
+  <si>
+    <t>Modular Liner Size MA/22 Elevated Wall  40+42</t>
+  </si>
+  <si>
+    <t>products/modular-liner-elevated-wall.png</t>
+  </si>
+  <si>
+    <t>MO-MLLE-MB/28 </t>
+  </si>
+  <si>
+    <t>Modular Liner Size MB/28 Elevated Wall  44 + 46</t>
+  </si>
+  <si>
+    <t>MO-MLLE-MD/32 </t>
+  </si>
+  <si>
+    <t>Modular Liner Size MD/32 Elevated Wall  48 + 50</t>
+  </si>
+  <si>
+    <t>MO-MLLE-MF/36 </t>
+  </si>
+  <si>
+    <t>Modular Liner Size MF/36 Elevated Wall  52 +54</t>
+  </si>
+  <si>
+    <t>MO-MLLE-MH/36 </t>
+  </si>
+  <si>
+    <t>Modular Liner Size MH/36 Elevated Wall  56 + 58</t>
+  </si>
+  <si>
+    <t>MO-MLLE-MJ/36 </t>
+  </si>
+  <si>
+    <t>Modular Liner Size MJ/36 Elevated Wall  60+ 62</t>
+  </si>
+  <si>
+    <t>MO-MSEC-40/MA</t>
+  </si>
+  <si>
+    <t>Cementless Modular Shell 40mm</t>
+  </si>
+  <si>
+    <t>products/cementless-modular-shell.png</t>
+  </si>
+  <si>
+    <t>MO-MSEC-42/MA</t>
+  </si>
+  <si>
+    <t>Cementless Modular Shell 42mm</t>
+  </si>
+  <si>
+    <t>MO-MSEC-44/MB</t>
+  </si>
+  <si>
+    <t>Cementless Modular Shell 44mm</t>
+  </si>
+  <si>
+    <t>MO-MSFC-46/MB</t>
+  </si>
+  <si>
+    <t>Cementless Modular Shell 46mm</t>
+  </si>
+  <si>
+    <t>MO-MSFC-48/MD</t>
+  </si>
+  <si>
+    <t>Cementless Modular Shell 48mm</t>
+  </si>
+  <si>
+    <t>MO-MSFC-50/MD</t>
+  </si>
+  <si>
+    <t>Cementless Modular Shell 50mm</t>
+  </si>
+  <si>
+    <t>MO-MSFC-52/MF</t>
+  </si>
+  <si>
+    <t>Cementless Modular Shell 52mm</t>
+  </si>
+  <si>
+    <t>MO-MSFC-54/MF</t>
+  </si>
+  <si>
+    <t>Cementless Modular Shell 54mm</t>
+  </si>
+  <si>
+    <t>MO-MSFC-56/MH</t>
+  </si>
+  <si>
+    <t>Cementless Modular Shell 56mm</t>
+  </si>
+  <si>
+    <t>MO-MSFC-58/MH</t>
+  </si>
+  <si>
+    <t>Cementless Modular Shell 58mm</t>
+  </si>
+  <si>
+    <t>MO-MSFC-60/MJ</t>
+  </si>
+  <si>
+    <t>Cementless Modular Shell 60mm</t>
+  </si>
+  <si>
+    <t>MO-MSFC-62/MJ</t>
+  </si>
+  <si>
+    <t>Cementless Modular Shell 62mm</t>
+  </si>
+  <si>
+    <t>MO-MSFC-64/MJ</t>
+  </si>
+  <si>
+    <t>Cementless Modular Shell 64mm</t>
+  </si>
+  <si>
+    <t>MO-MSFC-66/MK</t>
+  </si>
+  <si>
+    <t>Cementless Modular Shell 66mm</t>
+  </si>
+  <si>
+    <t>MO-MSFC-68/MK</t>
+  </si>
+  <si>
+    <t>Cementless Modular Shell 68mm</t>
+  </si>
+  <si>
+    <t>MO-MSFC-70/MK</t>
+  </si>
+  <si>
+    <t>Cementless Modular Shell 70mm</t>
+  </si>
+  <si>
+    <t>MO-STAC-25/01</t>
+  </si>
+  <si>
+    <t>Cementless Stem 130  Size 1 Standard 125°</t>
+  </si>
+  <si>
+    <t>products/cementless-stem-standard.png</t>
+  </si>
+  <si>
+    <t>MO-STAC-25/02</t>
+  </si>
+  <si>
+    <t>Cementless Stem 140  Size 2 Standard 125°</t>
+  </si>
+  <si>
+    <t>MO-STAC-25/03</t>
+  </si>
+  <si>
+    <t>Cementless Stem 145  Size 3 Standard 125°</t>
+  </si>
+  <si>
+    <t>MO-STAC-25/04</t>
+  </si>
+  <si>
+    <t>Cementless Stem 150  Size 4 Standard 125°</t>
+  </si>
+  <si>
+    <t>MO-STAC-25/05</t>
+  </si>
+  <si>
+    <t>Cementless Stem 154  Size 5 Standard 125°</t>
+  </si>
+  <si>
+    <t>MO-STAC-25/06</t>
+  </si>
+  <si>
+    <t>Cementless Stem 160  Size 6 Standard 125°</t>
+  </si>
+  <si>
+    <t>MO-STAC-25/07</t>
+  </si>
+  <si>
+    <t>Cementless Stem 165  Size 7 Standard 125°</t>
+  </si>
+  <si>
+    <t>MO-STAC-25/08</t>
+  </si>
+  <si>
+    <t>Cementless Stem 170  Size 8 Standard 125°</t>
+  </si>
+  <si>
+    <t>MO-STAC-25/09</t>
+  </si>
+  <si>
+    <t>Cementless Stem 180  Size 9 Standard 125°</t>
+  </si>
+  <si>
+    <t>MO-STAC-25/10</t>
+  </si>
+  <si>
+    <t>Cementless Stem 189  Size 10 Standard 125°</t>
+  </si>
+  <si>
+    <t>MO-STAC-35/00</t>
+  </si>
+  <si>
+    <t>Cementless Stem 115 Size 0 Standard 135°</t>
+  </si>
+  <si>
+    <t>MO-STAC-35/01</t>
+  </si>
+  <si>
+    <t>Cementless Stem 130 Size 1 Standard 135°</t>
+  </si>
+  <si>
+    <t>MO-STAC-35/02</t>
+  </si>
+  <si>
+    <t>Cementless Stem 140 Size 2 Standard 135°</t>
+  </si>
+  <si>
+    <t>MO-STAC-35/03</t>
+  </si>
+  <si>
+    <t>Cementless Stem 145 Size 3 Standard 135°</t>
+  </si>
+  <si>
+    <t>MO-STAC-35/04</t>
+  </si>
+  <si>
+    <t>Cementless Stem 150 Size 4 Standard 135°</t>
+  </si>
+  <si>
+    <t>MO-STAC-35/05</t>
+  </si>
+  <si>
+    <t>Cementless Stem 154 Size 5 Standard 135°</t>
+  </si>
+  <si>
+    <t>MO-STAC-35/06</t>
+  </si>
+  <si>
+    <t>Cementless Stem 160 Size 6 Standard 135°</t>
+  </si>
+  <si>
+    <t>MO-STAC-35/07</t>
+  </si>
+  <si>
+    <t>Cementless Stem 165 Size 7 Standard 135°</t>
+  </si>
+  <si>
+    <t>MO-STAC-35/08</t>
+  </si>
+  <si>
+    <t>Cementless Stem 170 Size 8 Standard 135°</t>
+  </si>
+  <si>
+    <t>MO-STAC-35/09</t>
+  </si>
+  <si>
+    <t>Cementless Stem 180 Size 9 Standard 135°</t>
+  </si>
+  <si>
+    <t>MO-STAC-35/10</t>
+  </si>
+  <si>
+    <t>Cementless Stem 189 Size 10 Standard 135°</t>
+  </si>
+  <si>
+    <t>MO-STBC-35/00</t>
+  </si>
+  <si>
+    <t>Cementless Stem 115 Size 0 Lateral 135°</t>
+  </si>
+  <si>
+    <t>products/cementless-stem-lateral.png</t>
+  </si>
+  <si>
+    <t>MO-STBC-35/01</t>
+  </si>
+  <si>
+    <t>Cementless Stem 130 Size 1 Lateral 135°</t>
+  </si>
+  <si>
+    <t>MO-STBC-35/02</t>
+  </si>
+  <si>
+    <t>Cementless Stem 140  Size 2 Lateral 135°</t>
+  </si>
+  <si>
+    <t>MO-STBC-35/03</t>
+  </si>
+  <si>
+    <t>Cementless Stem 145 Size 3 Lateral 135°</t>
+  </si>
+  <si>
+    <t>MO-STBC-35/04</t>
+  </si>
+  <si>
+    <t>Cementless Stem 150 Size 4 Lateral 135°</t>
+  </si>
+  <si>
+    <t>MO-STBC-35/05</t>
+  </si>
+  <si>
+    <t>Cementless Stem 154 Size 5 Lateral 135°</t>
+  </si>
+  <si>
+    <t>MO-STBC-35/06</t>
+  </si>
+  <si>
+    <t>Cementless Stem 160 Size 6 Lateral 135°</t>
+  </si>
+  <si>
+    <t>MO-STBC-35/07</t>
+  </si>
+  <si>
+    <t>Cementless Stem 165 Size 7 Lateral 135°</t>
+  </si>
+  <si>
+    <t>MO-STBC-35/08</t>
+  </si>
+  <si>
+    <t>Cementless Stem 170 Size 8 Lateral 135°</t>
+  </si>
+  <si>
+    <t>MO-STBC-35/09</t>
+  </si>
+  <si>
+    <t>Cementless Stem 180 Size 9 Lateral 135°</t>
+  </si>
+  <si>
+    <t>MO-STBC-35/10</t>
+  </si>
+  <si>
+    <t>Cementless Stem 189 Size 10 Lateral 135°</t>
+  </si>
+  <si>
+    <t>MO-STCM-00/00</t>
+  </si>
+  <si>
+    <t>Cemented Stem Standard 00 Offset 37mm</t>
+  </si>
+  <si>
+    <t>MO-STCM-00/01</t>
+  </si>
+  <si>
+    <t>Cemented Stem Standard 01 Offset 45mm</t>
+  </si>
+  <si>
+    <t>MO-STCM-00/02</t>
+  </si>
+  <si>
+    <t>Cemented Stem Standard 02 Offset 45mm</t>
+  </si>
+  <si>
+    <t>MO-STCM-00/03</t>
+  </si>
+  <si>
+    <t>Cemented Stem Standard 03 Offset 45mm</t>
+  </si>
+  <si>
+    <t>MO-STCM-00/04</t>
+  </si>
+  <si>
+    <t>Cemented Stem Standard 04 Offset 45mm</t>
+  </si>
+  <si>
+    <t>MO-STDM-00/01</t>
+  </si>
+  <si>
+    <t>Cemented Stem Narrow 01 Offset 38mm</t>
+  </si>
+  <si>
+    <t>MO-STDM-00/02</t>
+  </si>
+  <si>
+    <t>Cemented Stem Narrow 02 Offset 38mm</t>
+  </si>
+  <si>
+    <t>MO-STDM-00/03</t>
+  </si>
+  <si>
+    <t>Cemented Stem Narrow 03 Offset 38mm</t>
+  </si>
+  <si>
+    <t>MO-STDM-00/04</t>
+  </si>
+  <si>
+    <t>Cemented Stem Narrow 04 Offset 38mm</t>
+  </si>
+  <si>
+    <t>MO-SWCC-65/15</t>
+  </si>
+  <si>
+    <t>Bone Screw 6.5 mm X 15 mm</t>
+  </si>
+  <si>
+    <t>products/bone-screw.png</t>
+  </si>
+  <si>
+    <t>MO-SWCC-65/20</t>
+  </si>
+  <si>
+    <t>Bone Screw 6.5 mm X 20 mm</t>
+  </si>
+  <si>
+    <t>MO-SWCC-65/25</t>
+  </si>
+  <si>
+    <t>Bone Screw 6.5 mm X 25 mm</t>
+  </si>
+  <si>
+    <t>MO-SWCC-65/30</t>
+  </si>
+  <si>
+    <t>Bone Screw 6.5 mm X 30 mm</t>
+  </si>
+  <si>
+    <t>MO-SWCC-65/35</t>
+  </si>
+  <si>
+    <t>Bone Screw 6.5 mm X 35 mm</t>
+  </si>
+  <si>
+    <t>MO-SWCC-65/40</t>
+  </si>
+  <si>
+    <t>Bone Screw 6.5 mm X 40 mm</t>
+  </si>
+  <si>
+    <t>MO-SWCC-65/45</t>
+  </si>
+  <si>
+    <t>Bone Screw 6.5 mm X 45 mm</t>
+  </si>
+  <si>
+    <t>MO-SWCC-65/50</t>
+  </si>
+  <si>
+    <t>Bone Screw 6.5 mm X 50 mm</t>
+  </si>
+  <si>
+    <t>BCS1G40G</t>
+  </si>
+  <si>
+    <t>Bone Cement Synicem-1G_40g</t>
+  </si>
+  <si>
+    <t>manufacturer-008</t>
+  </si>
+  <si>
+    <t>products/Synicem-1G_40g.png</t>
   </si>
 </sst>
 </file>
@@ -1047,17 +1821,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H111"/>
+  <dimension ref="A1:H234"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.5703125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="42.42578125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="22.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="55.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="21.42578125" style="1" customWidth="1"/>
     <col min="5" max="5" width="15.85546875" style="1" customWidth="1"/>
     <col min="6" max="6" width="18.85546875" style="1" customWidth="1"/>
     <col min="7" max="7" width="5.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="32" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="64" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3286,6 +4060,2466 @@
         <v>234</v>
       </c>
     </row>
+    <row r="112" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A112" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="B112" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="D112" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E112" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F112" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H112" s="1" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="113" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A113" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="B113" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="D113" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E113" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F113" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H113" s="1" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="114" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A114" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="B114" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="D114" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E114" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F114" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H114" s="1" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="115" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A115" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B115" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="D115" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E115" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F115" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H115" s="1" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="116" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A116" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="B116" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="D116" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E116" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F116" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H116" s="1" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="117" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A117" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="B117" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="D117" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E117" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F117" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H117" s="1" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="118" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A118" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="B118" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="D118" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E118" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F118" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H118" s="1" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="119" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A119" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="B119" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="D119" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E119" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F119" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H119" s="1" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="120" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A120" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="B120" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="D120" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E120" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F120" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H120" s="1" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="121" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A121" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="B121" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="D121" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E121" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F121" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H121" s="1" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="122" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A122" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="B122" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="D122" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E122" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F122" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H122" s="1" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="123" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A123" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="B123" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="D123" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E123" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F123" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H123" s="1" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="124" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A124" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="B124" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="D124" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E124" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F124" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H124" s="1" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="125" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A125" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="B125" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="D125" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E125" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F125" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H125" s="1" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="126" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A126" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="B126" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="D126" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E126" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F126" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H126" s="1" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="127" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A127" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="B127" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="D127" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E127" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F127" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H127" s="1" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="128" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A128" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="B128" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="D128" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E128" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F128" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H128" s="1" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="129" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A129" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="B129" s="1" t="s">
+        <v>273</v>
+      </c>
+      <c r="D129" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E129" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F129" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H129" s="1" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="130" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A130" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="B130" s="1" t="s">
+        <v>275</v>
+      </c>
+      <c r="D130" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E130" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F130" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H130" s="1" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="131" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A131" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="B131" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="D131" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E131" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F131" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H131" s="1" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="132" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A132" s="1" t="s">
+        <v>279</v>
+      </c>
+      <c r="B132" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="D132" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E132" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F132" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H132" s="1" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="133" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A133" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="B133" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="D133" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E133" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F133" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H133" s="1" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="134" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A134" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="B134" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="D134" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E134" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F134" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H134" s="1" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="135" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A135" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="B135" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="D135" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E135" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F135" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H135" s="1" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="136" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A136" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="B136" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="D136" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E136" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F136" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H136" s="1" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="137" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A137" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="B137" s="1" t="s">
+        <v>290</v>
+      </c>
+      <c r="D137" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E137" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F137" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H137" s="1" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="138" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A138" s="1" t="s">
+        <v>291</v>
+      </c>
+      <c r="B138" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="D138" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E138" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F138" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H138" s="1" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="139" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A139" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="B139" s="1" t="s">
+        <v>294</v>
+      </c>
+      <c r="D139" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E139" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F139" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H139" s="1" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="140" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A140" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="B140" s="1" t="s">
+        <v>296</v>
+      </c>
+      <c r="D140" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E140" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F140" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H140" s="1" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="141" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A141" s="1" t="s">
+        <v>297</v>
+      </c>
+      <c r="B141" s="1" t="s">
+        <v>298</v>
+      </c>
+      <c r="D141" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E141" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F141" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H141" s="1" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="142" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A142" s="1" t="s">
+        <v>299</v>
+      </c>
+      <c r="B142" s="1" t="s">
+        <v>300</v>
+      </c>
+      <c r="D142" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E142" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F142" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H142" s="1" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="143" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A143" s="1" t="s">
+        <v>301</v>
+      </c>
+      <c r="B143" s="1" t="s">
+        <v>302</v>
+      </c>
+      <c r="D143" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E143" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F143" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H143" s="1" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="144" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A144" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="B144" s="1" t="s">
+        <v>304</v>
+      </c>
+      <c r="D144" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E144" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F144" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H144" s="1" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="145" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A145" s="1" t="s">
+        <v>305</v>
+      </c>
+      <c r="B145" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="D145" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E145" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F145" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H145" s="1" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="146" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A146" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="B146" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="D146" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E146" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F146" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H146" s="1" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="147" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A147" s="1" t="s">
+        <v>310</v>
+      </c>
+      <c r="B147" s="1" t="s">
+        <v>311</v>
+      </c>
+      <c r="D147" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E147" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F147" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H147" s="1" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="148" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A148" s="1" t="s">
+        <v>312</v>
+      </c>
+      <c r="B148" s="1" t="s">
+        <v>313</v>
+      </c>
+      <c r="D148" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E148" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F148" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H148" s="1" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="149" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A149" s="1" t="s">
+        <v>314</v>
+      </c>
+      <c r="B149" s="1" t="s">
+        <v>315</v>
+      </c>
+      <c r="D149" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E149" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F149" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H149" s="1" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="150" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A150" s="1" t="s">
+        <v>316</v>
+      </c>
+      <c r="B150" s="1" t="s">
+        <v>317</v>
+      </c>
+      <c r="D150" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E150" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F150" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H150" s="1" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="151" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A151" s="1" t="s">
+        <v>318</v>
+      </c>
+      <c r="B151" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="D151" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E151" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F151" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H151" s="1" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="152" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A152" s="1" t="s">
+        <v>320</v>
+      </c>
+      <c r="B152" s="1" t="s">
+        <v>321</v>
+      </c>
+      <c r="D152" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E152" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F152" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H152" s="1" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="153" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A153" s="1" t="s">
+        <v>322</v>
+      </c>
+      <c r="B153" s="1" t="s">
+        <v>323</v>
+      </c>
+      <c r="D153" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E153" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F153" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H153" s="1" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="154" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A154" s="1" t="s">
+        <v>324</v>
+      </c>
+      <c r="B154" s="1" t="s">
+        <v>325</v>
+      </c>
+      <c r="D154" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E154" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F154" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H154" s="1" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="155" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A155" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="B155" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="D155" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E155" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F155" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H155" s="1" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="156" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A156" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="B156" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="D156" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E156" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F156" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H156" s="1" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="157" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A157" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="B157" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="D157" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E157" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F157" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H157" s="1" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="158" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A158" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="B158" s="1" t="s">
+        <v>333</v>
+      </c>
+      <c r="D158" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E158" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F158" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H158" s="1" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="159" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A159" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="B159" s="1" t="s">
+        <v>335</v>
+      </c>
+      <c r="D159" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E159" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F159" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H159" s="1" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="160" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A160" s="1" t="s">
+        <v>336</v>
+      </c>
+      <c r="B160" s="1" t="s">
+        <v>337</v>
+      </c>
+      <c r="D160" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E160" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F160" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H160" s="1" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="161" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A161" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="B161" s="1" t="s">
+        <v>339</v>
+      </c>
+      <c r="D161" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E161" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F161" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H161" s="1" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="162" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A162" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="B162" s="1" t="s">
+        <v>341</v>
+      </c>
+      <c r="D162" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E162" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F162" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H162" s="1" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="163" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A163" s="1" t="s">
+        <v>342</v>
+      </c>
+      <c r="B163" s="1" t="s">
+        <v>343</v>
+      </c>
+      <c r="D163" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E163" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F163" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H163" s="1" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="164" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A164" s="1" t="s">
+        <v>345</v>
+      </c>
+      <c r="B164" s="1" t="s">
+        <v>346</v>
+      </c>
+      <c r="D164" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E164" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F164" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H164" s="1" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="165" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A165" s="1" t="s">
+        <v>347</v>
+      </c>
+      <c r="B165" s="1" t="s">
+        <v>348</v>
+      </c>
+      <c r="D165" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E165" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F165" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H165" s="1" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="166" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A166" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="B166" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="D166" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E166" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F166" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H166" s="1" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="167" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A167" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="B167" s="1" t="s">
+        <v>352</v>
+      </c>
+      <c r="D167" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E167" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F167" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H167" s="1" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="168" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A168" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="B168" s="1" t="s">
+        <v>354</v>
+      </c>
+      <c r="D168" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E168" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F168" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H168" s="1" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="169" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A169" s="1" t="s">
+        <v>355</v>
+      </c>
+      <c r="B169" s="1" t="s">
+        <v>356</v>
+      </c>
+      <c r="D169" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E169" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F169" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H169" s="1" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="170" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A170" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="B170" s="1" t="s">
+        <v>359</v>
+      </c>
+      <c r="D170" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E170" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F170" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H170" s="1" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="171" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A171" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="B171" s="1" t="s">
+        <v>361</v>
+      </c>
+      <c r="D171" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E171" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F171" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H171" s="1" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="172" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A172" s="1" t="s">
+        <v>362</v>
+      </c>
+      <c r="B172" s="1" t="s">
+        <v>363</v>
+      </c>
+      <c r="D172" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E172" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F172" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H172" s="1" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="173" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A173" s="1" t="s">
+        <v>364</v>
+      </c>
+      <c r="B173" s="1" t="s">
+        <v>365</v>
+      </c>
+      <c r="D173" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E173" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F173" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H173" s="1" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="174" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A174" s="1" t="s">
+        <v>366</v>
+      </c>
+      <c r="B174" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="D174" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E174" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F174" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H174" s="1" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="175" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A175" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="B175" s="1" t="s">
+        <v>369</v>
+      </c>
+      <c r="D175" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E175" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F175" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H175" s="1" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="176" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A176" s="1" t="s">
+        <v>370</v>
+      </c>
+      <c r="B176" s="1" t="s">
+        <v>371</v>
+      </c>
+      <c r="D176" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E176" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F176" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H176" s="1" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="177" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A177" s="1" t="s">
+        <v>372</v>
+      </c>
+      <c r="B177" s="1" t="s">
+        <v>373</v>
+      </c>
+      <c r="D177" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E177" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F177" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H177" s="1" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="178" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A178" s="1" t="s">
+        <v>374</v>
+      </c>
+      <c r="B178" s="1" t="s">
+        <v>375</v>
+      </c>
+      <c r="D178" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E178" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F178" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H178" s="1" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="179" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A179" s="1" t="s">
+        <v>376</v>
+      </c>
+      <c r="B179" s="1" t="s">
+        <v>377</v>
+      </c>
+      <c r="D179" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E179" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F179" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H179" s="1" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="180" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A180" s="1" t="s">
+        <v>378</v>
+      </c>
+      <c r="B180" s="1" t="s">
+        <v>379</v>
+      </c>
+      <c r="D180" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E180" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F180" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H180" s="1" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="181" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A181" s="1" t="s">
+        <v>380</v>
+      </c>
+      <c r="B181" s="1" t="s">
+        <v>381</v>
+      </c>
+      <c r="D181" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E181" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F181" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H181" s="1" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="182" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A182" s="1" t="s">
+        <v>382</v>
+      </c>
+      <c r="B182" s="1" t="s">
+        <v>383</v>
+      </c>
+      <c r="D182" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E182" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F182" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H182" s="1" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="183" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A183" s="1" t="s">
+        <v>384</v>
+      </c>
+      <c r="B183" s="1" t="s">
+        <v>385</v>
+      </c>
+      <c r="D183" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E183" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F183" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H183" s="1" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="184" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A184" s="1" t="s">
+        <v>386</v>
+      </c>
+      <c r="B184" s="1" t="s">
+        <v>387</v>
+      </c>
+      <c r="D184" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E184" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F184" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H184" s="1" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="185" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A185" s="1" t="s">
+        <v>388</v>
+      </c>
+      <c r="B185" s="1" t="s">
+        <v>389</v>
+      </c>
+      <c r="D185" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E185" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F185" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H185" s="1" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="186" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A186" s="1" t="s">
+        <v>391</v>
+      </c>
+      <c r="B186" s="1" t="s">
+        <v>392</v>
+      </c>
+      <c r="D186" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E186" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F186" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H186" s="1" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="187" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A187" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="B187" s="1" t="s">
+        <v>394</v>
+      </c>
+      <c r="D187" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E187" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F187" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H187" s="1" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="188" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A188" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="B188" s="1" t="s">
+        <v>396</v>
+      </c>
+      <c r="D188" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E188" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F188" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H188" s="1" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="189" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A189" s="1" t="s">
+        <v>397</v>
+      </c>
+      <c r="B189" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="D189" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E189" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F189" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H189" s="1" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="190" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A190" s="1" t="s">
+        <v>399</v>
+      </c>
+      <c r="B190" s="1" t="s">
+        <v>400</v>
+      </c>
+      <c r="D190" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E190" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F190" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H190" s="1" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="191" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A191" s="1" t="s">
+        <v>401</v>
+      </c>
+      <c r="B191" s="1" t="s">
+        <v>402</v>
+      </c>
+      <c r="D191" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E191" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F191" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H191" s="1" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="192" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A192" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="B192" s="1" t="s">
+        <v>404</v>
+      </c>
+      <c r="D192" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E192" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F192" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H192" s="1" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="193" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A193" s="1" t="s">
+        <v>405</v>
+      </c>
+      <c r="B193" s="1" t="s">
+        <v>406</v>
+      </c>
+      <c r="D193" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E193" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F193" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H193" s="1" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="194" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A194" s="1" t="s">
+        <v>407</v>
+      </c>
+      <c r="B194" s="1" t="s">
+        <v>408</v>
+      </c>
+      <c r="D194" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E194" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F194" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H194" s="1" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="195" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A195" s="1" t="s">
+        <v>409</v>
+      </c>
+      <c r="B195" s="1" t="s">
+        <v>410</v>
+      </c>
+      <c r="D195" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E195" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F195" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H195" s="1" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="196" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A196" s="1" t="s">
+        <v>411</v>
+      </c>
+      <c r="B196" s="1" t="s">
+        <v>412</v>
+      </c>
+      <c r="D196" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E196" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F196" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H196" s="1" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="197" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A197" s="1" t="s">
+        <v>413</v>
+      </c>
+      <c r="B197" s="1" t="s">
+        <v>414</v>
+      </c>
+      <c r="D197" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E197" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F197" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H197" s="1" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="198" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A198" s="1" t="s">
+        <v>415</v>
+      </c>
+      <c r="B198" s="1" t="s">
+        <v>416</v>
+      </c>
+      <c r="D198" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E198" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F198" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H198" s="1" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="199" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A199" s="1" t="s">
+        <v>417</v>
+      </c>
+      <c r="B199" s="1" t="s">
+        <v>418</v>
+      </c>
+      <c r="D199" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E199" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F199" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H199" s="1" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="200" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A200" s="1" t="s">
+        <v>419</v>
+      </c>
+      <c r="B200" s="1" t="s">
+        <v>420</v>
+      </c>
+      <c r="D200" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E200" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F200" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H200" s="1" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="201" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A201" s="1" t="s">
+        <v>421</v>
+      </c>
+      <c r="B201" s="1" t="s">
+        <v>422</v>
+      </c>
+      <c r="D201" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E201" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F201" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H201" s="1" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="202" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A202" s="1" t="s">
+        <v>423</v>
+      </c>
+      <c r="B202" s="1" t="s">
+        <v>424</v>
+      </c>
+      <c r="D202" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E202" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F202" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H202" s="1" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="203" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A203" s="1" t="s">
+        <v>425</v>
+      </c>
+      <c r="B203" s="1" t="s">
+        <v>426</v>
+      </c>
+      <c r="D203" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E203" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F203" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H203" s="1" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="204" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A204" s="1" t="s">
+        <v>427</v>
+      </c>
+      <c r="B204" s="1" t="s">
+        <v>428</v>
+      </c>
+      <c r="D204" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E204" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F204" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H204" s="1" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="205" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A205" s="1" t="s">
+        <v>429</v>
+      </c>
+      <c r="B205" s="1" t="s">
+        <v>430</v>
+      </c>
+      <c r="D205" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E205" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F205" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H205" s="1" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="206" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A206" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="B206" s="1" t="s">
+        <v>432</v>
+      </c>
+      <c r="D206" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E206" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F206" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H206" s="1" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="207" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A207" s="1" t="s">
+        <v>434</v>
+      </c>
+      <c r="B207" s="1" t="s">
+        <v>435</v>
+      </c>
+      <c r="D207" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E207" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F207" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H207" s="1" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="208" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A208" s="1" t="s">
+        <v>436</v>
+      </c>
+      <c r="B208" s="1" t="s">
+        <v>437</v>
+      </c>
+      <c r="D208" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E208" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F208" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H208" s="1" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="209" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A209" s="1" t="s">
+        <v>438</v>
+      </c>
+      <c r="B209" s="1" t="s">
+        <v>439</v>
+      </c>
+      <c r="D209" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E209" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F209" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H209" s="1" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="210" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A210" s="1" t="s">
+        <v>440</v>
+      </c>
+      <c r="B210" s="1" t="s">
+        <v>441</v>
+      </c>
+      <c r="D210" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E210" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F210" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H210" s="1" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="211" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A211" s="1" t="s">
+        <v>442</v>
+      </c>
+      <c r="B211" s="1" t="s">
+        <v>443</v>
+      </c>
+      <c r="D211" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E211" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F211" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H211" s="1" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="212" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A212" s="1" t="s">
+        <v>444</v>
+      </c>
+      <c r="B212" s="1" t="s">
+        <v>445</v>
+      </c>
+      <c r="D212" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E212" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F212" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H212" s="1" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="213" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A213" s="1" t="s">
+        <v>446</v>
+      </c>
+      <c r="B213" s="1" t="s">
+        <v>447</v>
+      </c>
+      <c r="D213" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E213" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F213" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H213" s="1" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="214" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A214" s="1" t="s">
+        <v>448</v>
+      </c>
+      <c r="B214" s="1" t="s">
+        <v>449</v>
+      </c>
+      <c r="D214" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E214" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F214" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H214" s="1" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="215" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A215" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="B215" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="D215" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E215" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F215" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H215" s="1" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="216" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A216" s="1" t="s">
+        <v>452</v>
+      </c>
+      <c r="B216" s="1" t="s">
+        <v>453</v>
+      </c>
+      <c r="D216" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E216" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F216" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H216" s="1" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="217" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A217" s="1" t="s">
+        <v>454</v>
+      </c>
+      <c r="B217" s="1" t="s">
+        <v>455</v>
+      </c>
+      <c r="D217" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E217" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F217" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H217" s="1" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="218" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A218" s="1" t="s">
+        <v>456</v>
+      </c>
+      <c r="B218" s="1" t="s">
+        <v>457</v>
+      </c>
+      <c r="D218" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E218" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F218" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H218" s="1" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="219" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A219" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="B219" s="1" t="s">
+        <v>459</v>
+      </c>
+      <c r="D219" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E219" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F219" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H219" s="1" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="220" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A220" s="1" t="s">
+        <v>460</v>
+      </c>
+      <c r="B220" s="1" t="s">
+        <v>461</v>
+      </c>
+      <c r="D220" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E220" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F220" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H220" s="1" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="221" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A221" s="1" t="s">
+        <v>462</v>
+      </c>
+      <c r="B221" s="1" t="s">
+        <v>463</v>
+      </c>
+      <c r="D221" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E221" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F221" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H221" s="1" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="222" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A222" s="1" t="s">
+        <v>464</v>
+      </c>
+      <c r="B222" s="1" t="s">
+        <v>465</v>
+      </c>
+      <c r="D222" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E222" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F222" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H222" s="1" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="223" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A223" s="1" t="s">
+        <v>466</v>
+      </c>
+      <c r="B223" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="D223" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E223" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F223" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H223" s="1" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="224" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A224" s="1" t="s">
+        <v>468</v>
+      </c>
+      <c r="B224" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="D224" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E224" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F224" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H224" s="1" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="225" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A225" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="B225" s="1" t="s">
+        <v>471</v>
+      </c>
+      <c r="D225" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E225" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F225" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H225" s="1" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="226" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A226" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="B226" s="1" t="s">
+        <v>473</v>
+      </c>
+      <c r="D226" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E226" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F226" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H226" s="1" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="227" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A227" s="1" t="s">
+        <v>475</v>
+      </c>
+      <c r="B227" s="1" t="s">
+        <v>476</v>
+      </c>
+      <c r="D227" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E227" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F227" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H227" s="1" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="228" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A228" s="1" t="s">
+        <v>477</v>
+      </c>
+      <c r="B228" s="1" t="s">
+        <v>478</v>
+      </c>
+      <c r="D228" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E228" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F228" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H228" s="1" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="229" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A229" s="1" t="s">
+        <v>479</v>
+      </c>
+      <c r="B229" s="1" t="s">
+        <v>480</v>
+      </c>
+      <c r="D229" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E229" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F229" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H229" s="1" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="230" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A230" s="1" t="s">
+        <v>481</v>
+      </c>
+      <c r="B230" s="1" t="s">
+        <v>482</v>
+      </c>
+      <c r="D230" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E230" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F230" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H230" s="1" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="231" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A231" s="1" t="s">
+        <v>483</v>
+      </c>
+      <c r="B231" s="1" t="s">
+        <v>484</v>
+      </c>
+      <c r="D231" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E231" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F231" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H231" s="1" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="232" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A232" s="1" t="s">
+        <v>485</v>
+      </c>
+      <c r="B232" s="1" t="s">
+        <v>486</v>
+      </c>
+      <c r="D232" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E232" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F232" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H232" s="1" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="233" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A233" s="1" t="s">
+        <v>487</v>
+      </c>
+      <c r="B233" s="1" t="s">
+        <v>488</v>
+      </c>
+      <c r="D233" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E233" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F233" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H233" s="1" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="234" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A234" s="1" t="s">
+        <v>489</v>
+      </c>
+      <c r="B234" s="1" t="s">
+        <v>490</v>
+      </c>
+      <c r="D234" s="1" t="s">
+        <v>491</v>
+      </c>
+      <c r="E234" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F234" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H234" s="1" t="s">
+        <v>492</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H111"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>